<commit_message>
Atualizações para leitura de horario e novos dados de metodos
</commit_message>
<xml_diff>
--- a/data/metodos.xlsx
+++ b/data/metodos.xlsx
@@ -44,9 +44,6 @@
     <t>Apostas / mês</t>
   </si>
   <si>
-    <t>Revalida</t>
-  </si>
-  <si>
     <t>Lay Zebra</t>
   </si>
   <si>
@@ -66,6 +63,9 @@
   </si>
   <si>
     <t>Limite LZ</t>
+  </si>
+  <si>
+    <t>BnR Lay Fora</t>
   </si>
 </sst>
 </file>
@@ -451,10 +451,10 @@
         <v>6</v>
       </c>
       <c r="B2" s="3">
-        <v>0.9</v>
+        <v>0.97</v>
       </c>
       <c r="C2" s="3">
-        <v>0.16</v>
+        <v>8.5000000000000006E-2</v>
       </c>
       <c r="D2" s="3">
         <v>1</v>
@@ -463,7 +463,7 @@
         <v>1</v>
       </c>
       <c r="F2" s="4">
-        <v>40</v>
+        <v>30</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -471,10 +471,10 @@
         <v>7</v>
       </c>
       <c r="B3" s="3">
-        <v>0.97</v>
+        <v>0.62</v>
       </c>
       <c r="C3" s="3">
-        <v>8.5000000000000006E-2</v>
+        <v>0.74</v>
       </c>
       <c r="D3" s="3">
         <v>1</v>
@@ -491,19 +491,19 @@
         <v>8</v>
       </c>
       <c r="B4" s="3">
-        <v>0.62</v>
+        <v>0.9</v>
       </c>
       <c r="C4" s="3">
-        <v>0.74</v>
+        <v>3.7999999999999999E-2</v>
       </c>
       <c r="D4" s="3">
-        <v>1</v>
+        <v>0.09</v>
       </c>
       <c r="E4" s="3">
-        <v>1</v>
+        <v>0.15</v>
       </c>
       <c r="F4" s="4">
-        <v>30</v>
+        <v>45</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -511,19 +511,19 @@
         <v>9</v>
       </c>
       <c r="B5" s="3">
-        <v>0.7</v>
+        <v>0.97</v>
       </c>
       <c r="C5" s="3">
         <v>0.06</v>
       </c>
       <c r="D5" s="3">
-        <v>7.4999999999999997E-2</v>
+        <v>1</v>
       </c>
       <c r="E5" s="3">
-        <v>0.15</v>
+        <v>1</v>
       </c>
       <c r="F5" s="4">
-        <v>35</v>
+        <v>30</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -531,10 +531,10 @@
         <v>10</v>
       </c>
       <c r="B6" s="3">
-        <v>0.97</v>
+        <v>0.95</v>
       </c>
       <c r="C6" s="3">
-        <v>0.06</v>
+        <v>7.6999999999999999E-2</v>
       </c>
       <c r="D6" s="3">
         <v>1</v>
@@ -551,10 +551,10 @@
         <v>11</v>
       </c>
       <c r="B7" s="3">
-        <v>0.95</v>
+        <v>0.97499999999999998</v>
       </c>
       <c r="C7" s="3">
-        <v>7.6999999999999999E-2</v>
+        <v>4.4444444444444446E-2</v>
       </c>
       <c r="D7" s="3">
         <v>1</v>
@@ -567,14 +567,14 @@
       </c>
     </row>
     <row r="8" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="2" t="s">
+      <c r="A8" s="5" t="s">
         <v>12</v>
       </c>
       <c r="B8" s="3">
-        <v>0.97499999999999998</v>
+        <v>0.8</v>
       </c>
       <c r="C8" s="3">
-        <v>4.4444444444444446E-2</v>
+        <v>0.28999999999999998</v>
       </c>
       <c r="D8" s="3">
         <v>1</v>
@@ -583,7 +583,7 @@
         <v>1</v>
       </c>
       <c r="F8" s="4">
-        <v>30</v>
+        <v>60</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -591,10 +591,10 @@
         <v>13</v>
       </c>
       <c r="B9" s="3">
-        <v>0.8</v>
+        <v>0.94</v>
       </c>
       <c r="C9" s="3">
-        <v>0.28999999999999998</v>
+        <v>0.09</v>
       </c>
       <c r="D9" s="3">
         <v>1</v>
@@ -603,7 +603,7 @@
         <v>1</v>
       </c>
       <c r="F9" s="4">
-        <v>60</v>
+        <v>30</v>
       </c>
     </row>
   </sheetData>

</xml_diff>